<commit_message>
Merge working offline with outdated online
</commit_message>
<xml_diff>
--- a/excel_templates/Backup_NTA_Template.xlsx
+++ b/excel_templates/Backup_NTA_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samscott/Desktop/NTAWeb/excel_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE053FE7-74E6-054B-9EF9-9EF26267A783}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32919D10-B6C8-2E42-B98A-A03A18449835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{89CE6B3D-78DD-D94C-B005-DB023AC169C8}"/>
   </bookViews>
@@ -33,6 +33,28 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -789,15 +811,6 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -824,6 +837,15 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1175,48 +1197,48 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="68" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60"/>
-      <c r="I2" s="60"/>
-      <c r="J2" s="60"/>
-      <c r="K2" s="60"/>
-      <c r="L2" s="60"/>
-      <c r="M2" s="61"/>
-      <c r="P2" s="59" t="s">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="60"/>
-      <c r="R2" s="60"/>
-      <c r="S2" s="61"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="70"/>
+      <c r="P2" s="68" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="69"/>
+      <c r="R2" s="69"/>
+      <c r="S2" s="70"/>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B3" s="59" t="s">
+      <c r="B3" s="68" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="60"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="59" t="s">
+      <c r="C3" s="69"/>
+      <c r="D3" s="70"/>
+      <c r="E3" s="68" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="60"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="59" t="s">
+      <c r="F3" s="69"/>
+      <c r="G3" s="70"/>
+      <c r="H3" s="68" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="60"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="59" t="s">
+      <c r="I3" s="69"/>
+      <c r="J3" s="70"/>
+      <c r="K3" s="68" t="s">
         <v>10</v>
       </c>
-      <c r="L3" s="60"/>
-      <c r="M3" s="61"/>
+      <c r="L3" s="69"/>
+      <c r="M3" s="70"/>
       <c r="P3" s="2" t="str">
         <f>B3</f>
         <v>Empty</v>
@@ -1238,26 +1260,26 @@
       <c r="A4" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="62" t="s">
+      <c r="B4" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="63"/>
-      <c r="D4" s="64"/>
-      <c r="E4" s="62" t="s">
+      <c r="C4" s="60"/>
+      <c r="D4" s="61"/>
+      <c r="E4" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="63"/>
-      <c r="G4" s="64"/>
-      <c r="H4" s="62" t="s">
+      <c r="F4" s="60"/>
+      <c r="G4" s="61"/>
+      <c r="H4" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="I4" s="63"/>
-      <c r="J4" s="64"/>
-      <c r="K4" s="62" t="s">
+      <c r="I4" s="60"/>
+      <c r="J4" s="61"/>
+      <c r="K4" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="L4" s="63"/>
-      <c r="M4" s="64"/>
+      <c r="L4" s="60"/>
+      <c r="M4" s="61"/>
       <c r="P4" s="5" t="str">
         <f>B4</f>
         <v>Empty</v>
@@ -1567,53 +1589,137 @@
       <c r="A14" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B14" s="24" t="str">
-        <f>IFERROR((P19-INDEX(B5:B12,P14))/(INDEX(B5:B12,P14+1)-INDEX(B5:B12,P14))*(INDEX(A5:A12,P14+1)-INDEX(A5:A12,P14))+INDEX(A5:A12,P14), "≤" &amp; A5)</f>
-        <v>≤50</v>
-      </c>
-      <c r="C14" s="24" t="str">
-        <f>IFERROR((Q19-INDEX(C5:C12,Q14))/(INDEX(C5:C12,Q14+1)-INDEX(C5:C12,Q14))*(INDEX(A5:A12,Q14+1)-INDEX(A5:A12,Q14))+INDEX(A5:A12,Q14), "≤" &amp; A5)</f>
-        <v>≤50</v>
-      </c>
-      <c r="D14" s="24" t="str">
-        <f>IFERROR((R19-INDEX(D5:D12,R14))/(INDEX(D5:D12,R14+1)-INDEX(D5:D12,R14))*(INDEX(A5:A12,R14+1)-INDEX(A5:A12,R14))+INDEX(A5:A12,R14), "≤" &amp; A5)</f>
-        <v>≤50</v>
-      </c>
-      <c r="E14" s="24" t="str">
-        <f>IFERROR((S19-INDEX(E5:E12,S14))/(INDEX(E5:E12,S14+1)-INDEX(E5:E12,S14))*(INDEX(A5:A12,S14+1)-INDEX(A5:A12,S14))+INDEX(A5:A12,S14), "≤" &amp; A5)</f>
-        <v>≤50</v>
-      </c>
-      <c r="F14" s="24" t="str">
-        <f>IFERROR((T19-INDEX(F5:F12,T14))/(INDEX(F5:F12,T14+1)-INDEX(F5:F12,T14))*(INDEX(A5:A12,T14+1)-INDEX(A5:A12,T14))+INDEX(A5:A12,T14), "≤" &amp; A5)</f>
-        <v>≤50</v>
-      </c>
-      <c r="G14" s="24" t="str">
-        <f>IFERROR((U19-INDEX(G5:G12,U14))/(INDEX(G5:G12,U14+1)-INDEX(G5:G12,U14))*(INDEX(A5:A12,U14+1)-INDEX(A5:A12,U14))+INDEX(A5:A12,U14), "≤" &amp; A5)</f>
-        <v>≤50</v>
-      </c>
-      <c r="H14" s="24" t="str">
-        <f>IFERROR((V19-INDEX(H5:H12,V14))/(INDEX(H5:H12,V14+1)-INDEX(H5:H12,V14))*(INDEX(A5:A12,V14+1)-INDEX(A5:A12,V14))+INDEX(A5:A12,V14), "≤" &amp; A5)</f>
-        <v>≤50</v>
-      </c>
-      <c r="I14" s="24" t="str">
-        <f>IFERROR((W19-INDEX(I5:I12,W14))/(INDEX(I5:I12,W14+1)-INDEX(I5:I12,W14))*(INDEX(A5:A12,W14+1)-INDEX(A5:A12,W14))+INDEX(A5:A12,W14), "≤" &amp; A5)</f>
-        <v>≤50</v>
-      </c>
-      <c r="J14" s="24" t="str">
-        <f>IFERROR((X19-INDEX(J5:J12,X14))/(INDEX(J5:J12,X14+1)-INDEX(J5:J12,X14))*(INDEX(A5:A12,X14+1)-INDEX(A5:A12,X14))+INDEX(A5:A12,X14), "≤" &amp; A5)</f>
-        <v>≤50</v>
-      </c>
-      <c r="K14" s="24" t="str">
-        <f>IFERROR((Y19-INDEX(K5:K12,Y14))/(INDEX(K5:K12,Y14+1)-INDEX(K5:K12,Y14))*(INDEX(A5:A12,Y14+1)-INDEX(A5:A12,Y14))+INDEX(A5:A12,Y14), "≤" &amp; A5)</f>
-        <v>≤50</v>
-      </c>
-      <c r="L14" s="24" t="str">
-        <f>IFERROR((Z19-INDEX(L5:L12,Z14))/(INDEX(L5:L12,Z14+1)-INDEX(L5:L12,Z14))*(INDEX(A5:A12,Z14+1)-INDEX(A5:A12,Z14))+INDEX(A5:A12,Z14), "≤" &amp; A5)</f>
-        <v>≤50</v>
-      </c>
-      <c r="M14" s="25" t="str">
-        <f>IFERROR((AA19-INDEX(M5:M12,AA14))/(INDEX(M5:M12,AA14+1)-INDEX(M5:M12,AA14))*(INDEX(A5:A12,AA14+1)-INDEX(A5:A12,AA14))+INDEX(A5:A12,AA14), "≤" &amp; A5)</f>
-        <v>≤50</v>
+      <c r="B14" s="24" t="e" cm="1">
+        <f t="array" ref="B14">IF(
+    (P19-INDEX(B5:B12,P14))/
+    (INDEX(B5:B12,P14+1)-INDEX(B5:B12,P14))*
+    (INDEX(A5:A12,P14+1)-INDEX(A5:A12,P14))+
+    INDEX(A5:A12,P14) &gt; A11,
+    "≥"&amp;A11,
+    "≤"&amp;A5
+)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C14" s="24" t="e" cm="1">
+        <f t="array" ref="C14">IF(
+    (Q19-INDEX(C5:C12,Q14))/
+    (INDEX(C5:C12,Q14+1)-INDEX(C5:C12,Q14))*
+    (INDEX(A5:A12,Q14+1)-INDEX(A5:A12,Q14))+
+    INDEX(A5:A12,Q14) &gt; A11,
+    "≥"&amp;A11,
+    "≤"&amp;A5
+)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D14" s="24" t="e" cm="1">
+        <f t="array" ref="D14">IF(
+    (R19-INDEX(D5:D12,R14))/
+    (INDEX(D5:D12,R14+1)-INDEX(D5:D12,R14))*
+    (INDEX(A5:A12,R14+1)-INDEX(A5:A12,R14))+
+    INDEX(A5:A12,R14) &gt; A11,
+    "≥"&amp;A11,
+    "≤"&amp;A5
+)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E14" s="24" t="e" cm="1">
+        <f t="array" ref="E14">IF(
+    (S19-INDEX(E5:E12,S14))/
+    (INDEX(E5:E12,S14+1)-INDEX(E5:E12,S14))*
+    (INDEX(A5:A12,S14+1)-INDEX(A5:A12,S14))+
+    INDEX(A5:A12,S14) &gt; A11,
+    "≥"&amp;A11,
+    "≤"&amp;A5
+)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F14" s="24" t="e" cm="1">
+        <f t="array" ref="F14">IF(
+    (T19-INDEX(F5:F12,T14))/
+    (INDEX(F5:F12,T14+1)-INDEX(F5:F12,T14))*
+    (INDEX(A5:A12,T14+1)-INDEX(A5:A12,T14))+
+    INDEX(A5:A12,T14) &gt; A11,
+    "≥"&amp;A11,
+    "≤"&amp;A5
+)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G14" s="24" t="e" cm="1">
+        <f t="array" ref="G14">IF(
+    (U19-INDEX(G5:G12,U14))/
+    (INDEX(G5:G12,U14+1)-INDEX(G5:G12,U14))*
+    (INDEX(A5:A12,U14+1)-INDEX(A5:A12,U14))+
+    INDEX(A5:A12,U14) &gt; A11,
+    "≥"&amp;A11,
+    "≤"&amp;A5
+)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H14" s="24" t="e" cm="1">
+        <f t="array" ref="H14">IF(
+    (V19-INDEX(H5:H12,V14))/
+    (INDEX(H5:H12,V14+1)-INDEX(H5:H12,V14))*
+    (INDEX(A5:A12,V14+1)-INDEX(A5:A12,V14))+
+    INDEX(A5:A12,V14) &gt; A11,
+    "≥"&amp;A11,
+    "≤"&amp;A5
+)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I14" s="24" t="e" cm="1">
+        <f t="array" ref="I14">IF(
+    (W19-INDEX(I5:I12,W14))/
+    (INDEX(I5:I12,W14+1)-INDEX(I5:I12,W14))*
+    (INDEX(A5:A12,W14+1)-INDEX(A5:A12,W14))+
+    INDEX(A5:A12,W14) &gt; A11,
+    "≥"&amp;A11,
+    "≤"&amp;A5
+)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J14" s="24" t="e" cm="1">
+        <f t="array" ref="J14">IF(
+    (X19-INDEX(J5:J12,X14))/
+    (INDEX(J5:J12,X14+1)-INDEX(J5:J12,X14))*
+    (INDEX(A5:A12,X14+1)-INDEX(A5:A12,X14))+
+    INDEX(A5:A12,X14) &gt; A11,
+    "≥"&amp;A11,
+    "≤"&amp;A5
+)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K14" s="24" t="e" cm="1">
+        <f t="array" ref="K14">IF(
+    (Y19-INDEX(K5:K12,Y14))/
+    (INDEX(K5:K12,Y14+1)-INDEX(K5:K12,Y14))*
+    (INDEX(A5:A12,Y14+1)-INDEX(A5:A12,Y14))+
+    INDEX(A5:A12,Y14) &gt; A11,
+    "≥"&amp;A11,
+    "≤"&amp;A5
+)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L14" s="24" t="e" cm="1">
+        <f t="array" ref="L14">IF(
+    (Z19-INDEX(L5:L12,Z14))/
+    (INDEX(L5:L12,Z14+1)-INDEX(L5:L12,Z14))*
+    (INDEX(A5:A12,Z14+1)-INDEX(A5:A12,Z14))+
+    INDEX(A5:A12,Z14) &gt; A11,
+    "≥"&amp;A11,
+    "≤"&amp;A5
+)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="M14" s="25" t="e" cm="1">
+        <f t="array" ref="M14">IF(
+    (AA19-INDEX(M5:M12,AA14))/
+    (INDEX(M5:M12,AA14+1)-INDEX(M5:M12,AA14))*
+    (INDEX(A5:A12,AA14+1)-INDEX(A5:A12,AA14))+
+    INDEX(A5:A12,AA14) &gt; A11,
+    "≥"&amp;A11,
+    "≤"&amp;A5
+)</f>
+        <v>#N/A</v>
       </c>
       <c r="O14" s="37" t="s">
         <v>13</v>
@@ -1688,17 +1794,38 @@
       <c r="A16" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B16" s="26" t="str">
-        <f>IFERROR((P21-INDEX(B5:B12,P16))/(INDEX(B5:B12,P16+1)-INDEX(B5:B12,P16))*(INDEX(A5:A12,P16+1)-INDEX(A5:A12,P16))+INDEX(A5:A12,P16), "≤" &amp; A5)</f>
-        <v>≤50</v>
-      </c>
-      <c r="C16" s="26" t="str">
-        <f>IFERROR((Q21-INDEX(C5:C12,Q16))/(INDEX(C5:C12,Q16+1)-INDEX(C5:C12,Q16))*(INDEX(A5:A12,Q16+1)-INDEX(A5:A12,Q16))+INDEX(A5:A12,Q16), "≤" &amp; A5)</f>
-        <v>≤50</v>
-      </c>
-      <c r="D16" s="26" t="str">
-        <f>IFERROR((R21-INDEX(D5:D12,R16))/(INDEX(D5:D12,R16+1)-INDEX(D5:D12,R16))*(INDEX(A5:A12,R16+1)-INDEX(A5:A12,R16))+INDEX(A5:A12,R16), "≤" &amp; A5)</f>
-        <v>≤50</v>
+      <c r="B16" s="26" t="e" cm="1">
+        <f t="array" ref="B16">IF(
+    (P21-INDEX(B5:B12,P16))/
+    (INDEX(B5:B12,P16+1)-INDEX(B5:B12,P16))*
+    (INDEX(A5:A12,P16+1)-INDEX(A5:A12,P16))+
+    INDEX(A5:A12,P16) &gt; A11,
+    "≥"&amp;A11,
+    "≤"&amp;A5
+)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C16" s="26" t="e" cm="1">
+        <f t="array" ref="C16">IF(
+    (Q21-INDEX(B5:B12,Q16))/
+    (INDEX(B5:B12,Q16+1)-INDEX(B5:B12,Q16))*
+    (INDEX(A5:A12,Q16+1)-INDEX(A5:A12,Q16))+
+    INDEX(A5:A12,Q16) &gt; A11,
+    "≥"&amp;A11,
+    "≤"&amp;A5
+)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D16" s="26" t="e" cm="1">
+        <f t="array" ref="D16">IF(
+    (R21-INDEX(D5:D12,R16))/
+    (INDEX(D5:D12,R16+1)-INDEX(D5:D12,R16))*
+    (INDEX(A5:A12,R16+1)-INDEX(A5:A12,R16))+
+    INDEX(A5:A12,R16) &gt; A11,
+    "≥"&amp;A11,
+    "≤"&amp;A5
+)</f>
+        <v>#N/A</v>
       </c>
       <c r="E16" s="26" t="str">
         <f>IFERROR((S21-INDEX(E5:E12,S16))/(INDEX(E5:E12,S16+1)-INDEX(E5:E12,S16))*(INDEX(A5:A12,S16+1)-INDEX(A5:A12,S16))+INDEX(A5:A12,S16), "≤" &amp; A5)</f>
@@ -1826,27 +1953,55 @@
         <v>5</v>
       </c>
       <c r="B19" s="45"/>
-      <c r="C19" s="46" t="str">
-        <f>IFERROR(AVERAGE(B14:D14), "≤" &amp; A5)</f>
-        <v>≤50</v>
+      <c r="C19" s="46" t="e">
+        <f>_xlfn.LET(
+    _xlpm.x, AVERAGE(B14:D14),
+    IF(_xlpm.x &lt;= A5, "≤"&amp;A5,
+        IF(_xlpm.x &gt;= A11, "≥"&amp;A11,
+            _xlpm.x
+        )
+    )
+)</f>
+        <v>#N/A</v>
       </c>
       <c r="D19" s="47"/>
       <c r="E19" s="45"/>
-      <c r="F19" s="46" t="str">
-        <f>IFERROR(AVERAGE(E14:G14), "≤" &amp; A5)</f>
-        <v>≤50</v>
+      <c r="F19" s="46" t="e">
+        <f>_xlfn.LET(
+    _xlpm.x, AVERAGE(E14:G14),
+    IF(_xlpm.x &lt;= A5, "≤"&amp;A5,
+        IF(_xlpm.x &gt;= A11, "≥"&amp;A11,
+            _xlpm.x
+        )
+    )
+)</f>
+        <v>#N/A</v>
       </c>
       <c r="G19" s="48"/>
       <c r="H19" s="45"/>
-      <c r="I19" s="46" t="str">
-        <f>IFERROR(AVERAGE(H14:J14), "≤" &amp; A5)</f>
-        <v>≤50</v>
+      <c r="I19" s="46" t="e">
+        <f>_xlfn.LET(
+    _xlpm.x, AVERAGE(H14:J14),
+    IF(_xlpm.x &lt;= A5, "≤"&amp;A5,
+        IF(_xlpm.x &gt;= A11, "≥"&amp;A11,
+            _xlpm.x
+        )
+    )
+)</f>
+        <v>#N/A</v>
       </c>
       <c r="J19" s="48"/>
       <c r="K19" s="45"/>
-      <c r="L19" s="46" t="str">
-        <f>IFERROR(AVERAGE(K14:M14), "≤" &amp; A5)</f>
-        <v>≤50</v>
+      <c r="L19" s="46" t="e">
+        <f>_xlfn.LET(
+    _xlpm.x, AVERAGE(K14:M14),
+    IF(_xlpm.x &lt;= A5, "≤"&amp;A5,
+        IF(_xlpm.x &gt;= A11, "≥"&amp;A11,
+            _xlpm.x
+        )
+    )
+)</f>
+        <v>#N/A</v>
       </c>
       <c r="M19" s="48"/>
       <c r="O19" s="41" t="s">
@@ -1998,20 +2153,20 @@
       </c>
     </row>
     <row r="24" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="F24" s="65" t="s">
+      <c r="F24" s="62" t="s">
         <v>8</v>
       </c>
-      <c r="G24" s="67" t="s">
+      <c r="G24" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="H24" s="69" t="s">
+      <c r="H24" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="I24" s="70"/>
+      <c r="I24" s="67"/>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="F25" s="66"/>
-      <c r="G25" s="68"/>
+      <c r="F25" s="63"/>
+      <c r="G25" s="65"/>
       <c r="H25" s="18" t="s">
         <v>2</v>
       </c>
@@ -2028,12 +2183,12 @@
         <f>$B$4</f>
         <v>Empty</v>
       </c>
-      <c r="H26" s="15" t="str">
+      <c r="H26" s="15" t="e">
         <f>IF(ISNUMBER(C19),
     IF(C19 &lt; A5, "≤" &amp; A5, IF(C19 &gt; A11, "≥" &amp; A11, C19)),
     IF(VALUE(SUBSTITUTE(C19, "≤", "")) &lt; A5, "≤" &amp; A5, C19)
 )</f>
-        <v>≤50</v>
+        <v>#N/A</v>
       </c>
       <c r="I26" s="21" t="str">
         <f>IF(ISNUMBER(C21),
@@ -2052,9 +2207,9 @@
         <f>$E$4</f>
         <v>Empty</v>
       </c>
-      <c r="H27" s="16" t="str">
+      <c r="H27" s="16" t="e">
         <f>IF(ISNUMBER(F19), IF(F19 &lt; A5, "≤" &amp; A5, IF(F19 &gt; A11, "≥" &amp; A11, F19)), IF(VALUE(SUBSTITUTE(F19, "≤", "")) &lt; A5, "≤" &amp; A5, F19) )</f>
-        <v>≤50</v>
+        <v>#N/A</v>
       </c>
       <c r="I27" s="22" t="str">
         <f>IF(ISNUMBER(F21),
@@ -2073,12 +2228,12 @@
         <f>$H$4</f>
         <v>Empty</v>
       </c>
-      <c r="H28" s="16" t="str">
+      <c r="H28" s="16" t="e">
         <f>IF(ISNUMBER(I19),
     IF(I19 &lt; A5, "≤" &amp; A5, IF(I19 &gt; A11, "≥" &amp; A11, I19)),
     IF(VALUE(SUBSTITUTE(I19, "≤", "")) &lt; A5, "≤" &amp; A5, I19)
 )</f>
-        <v>≤50</v>
+        <v>#N/A</v>
       </c>
       <c r="I28" s="22" t="str">
         <f>IF(ISNUMBER(I21),
@@ -2097,12 +2252,12 @@
         <f>$K$4</f>
         <v>Empty</v>
       </c>
-      <c r="H29" s="17" t="str">
+      <c r="H29" s="17" t="e">
         <f>IF(ISNUMBER(L19),
     IF(L19 &lt; A5, "≤" &amp; A5, IF(L19 &gt; A11, "≥" &amp; A11, L19)),
     IF(VALUE(SUBSTITUTE(L19, "≤", "")) &lt; A5, "≤" &amp; A5, L19)
 )</f>
-        <v>≤50</v>
+        <v>#N/A</v>
       </c>
       <c r="I29" s="23" t="str">
         <f>IF(ISNUMBER(L21),
@@ -2124,6 +2279,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="P2:S2"/>
+    <mergeCell ref="B2:M2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="K3:M3"/>
     <mergeCell ref="K4:M4"/>
     <mergeCell ref="H4:J4"/>
     <mergeCell ref="E4:G4"/>
@@ -2131,12 +2292,6 @@
     <mergeCell ref="F24:F25"/>
     <mergeCell ref="G24:G25"/>
     <mergeCell ref="H24:I24"/>
-    <mergeCell ref="P2:S2"/>
-    <mergeCell ref="B2:M2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="K3:M3"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="B5:M12">

</xml_diff>